<commit_message>
Never impute the diagnosis gates
dx_diabetes and dx_cholesterol carried na_rule = implied:0, so a gate left
unanswered was filled with zero and the respondent silently declared
undiagnosed. Both are now mar, matching dx_hypertension: rows with an
undefined gate drop and are counted in the attrition file.

Verified against the real file. Diabetes 7,851 -> 6,832 (3.8%), cholesterol
7,244 -> 5,944 (32.0%), hypertension unchanged at 6,346 (15.2%), which are
the cohorts reported to the group on 15/09/2026. The notes sheet records the
change.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pipeline/PNS_preprocessing_registry_v1.xlsx
+++ b/pipeline/PNS_preprocessing_registry_v1.xlsx
@@ -3812,7 +3812,7 @@
       <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>implied:0</t>
+          <t>mar</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -3932,7 +3932,7 @@
       <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>implied:0</t>
+          <t>mar</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -7405,7 +7405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7670,6 +7670,21 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Diagnosis gates</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>dx_diabetes and dx_cholesterol carried na_rule = implied:0, so an unanswered gate was filled with zero and the row declared undiagnosed. That is bug 1 of the 15/09/2026 build note and it builds 7,851 and 7,244 rows. Set to mar on 22/09/2026, matching dx_hypertension: the cohorts are now 6,832 (3.8%) and 5,944 (32.0%), as reported.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>